<commit_message>
Keep screen wiring unchanged, use software serial for DL-20
Screen (LCD+touch) wiring completely unchanged:

- LCD: PB0-PB15, PC4-PC7, PD2 (unchanged)

- Touch: PC8-PC12 (unchanged)

Lock end conflict resolution (no screen changes):

- DL-20 moved to software serial on PA0(TX)/PA1(RX) at 9600 baud

- DIP switch moved to PC0/PC2/PC3/PA8 (all free pins)

- Status LED moved to PA15 (JTAG disabled, SWD only)

- CH340 stays on USART1, UWB base stays on USART2

Fixed LQFP64 issue: only PD0/PD1/PD2 exist, no PD3-PD15

Key end: no changes, all hardware USART, no conflicts
</commit_message>
<xml_diff>
--- a/Doc/硬件引脚分配表.xlsx
+++ b/Doc/硬件引脚分配表.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -627,14 +627,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>野火STM32F103_MINI 智能门锁端 硬件接线表（冲突已解决）</t>
+          <t>野火STM32F103_MINI 智能门锁端 硬件接线表（屏幕不动，无冲突）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>芯片: STM32F103RCT6 (LQFP64) | 板载LCD+触摸屏+SPI Flash+蜂鸣器 | 外接UWB基站+DL-20+拨码开关 | 无引脚冲突</t>
+          <t>STM32F103RCT6 LQFP64(仅PD0/PD1/PD2) | LCD+触摸屏接线完全不动 | DL-20用软件串口 | 所有硬件USART不冲突</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>AMS1117-3.3 LDO输出</t>
+          <t>AMS1117-3.3 LDO</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>BOOT0引脚</t>
+          <t>BOOT0</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>SWD调试接口</t>
+          <t>SWD调试</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>SWD调试接口</t>
+          <t>SWD调试</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -913,7 +913,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>二、板载LCD (ILI9341) — 16位8080并口占整个GPIOB</t>
+          <t>二、板载LCD (ILI9341) — 接线完全不动</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
@@ -931,17 +931,17 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>PB0~PB7</t>
+          <t>PB0~PB15</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>LCD-D0~D7</t>
+          <t>LCD-D0~D15</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>LCD数据低8位</t>
+          <t>LCD 16位数据</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -951,12 +951,12 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>✅ LCD必须使用，LED放弃板载LED</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>8080数据线[0:7]</t>
+          <t>8080并口，占整个GPIOB</t>
         </is>
       </c>
     </row>
@@ -968,17 +968,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>PB8~PB15</t>
+          <t>PC4</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>LCD-D8~D15</t>
+          <t>LCD-CS</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>LCD数据高8位</t>
+          <t>LCD片选</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -988,12 +988,12 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>8080数据线[8:15]</t>
+          <t>低电平有效</t>
         </is>
       </c>
     </row>
@@ -1005,17 +1005,17 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>PC5</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>LCD-CS</t>
+          <t>LCD-RD</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>LCD片选</t>
+          <t>LCD读使能</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -1042,17 +1042,17 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>PC5</t>
+          <t>PC6</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>LCD-RD</t>
+          <t>LCD-WR</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>LCD读使能</t>
+          <t>LCD写使能</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1079,17 +1079,17 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>PC6</t>
+          <t>PC7</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>LCD-WR</t>
+          <t>LCD-DC</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>LCD写使能</t>
+          <t>LCD数据/命令</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>低电平有效</t>
+          <t>0=命令,1=数据</t>
         </is>
       </c>
     </row>
@@ -1116,17 +1116,17 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>PC7</t>
+          <t>PD2</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>LCD-DC</t>
+          <t>LCD-BL</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>LCD数据/命令</t>
+          <t>LCD背光</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -1136,262 +1136,262 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>0=命令,1=数据</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+          <t>高电平点亮</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>三、板载触摸屏 (XPT2046) — 接线完全不动</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>PD2</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>LCD-BL</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>LCD背光控制</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>PC8</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>TP-CLK</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>触摸SPI时钟</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>高电平点亮背光</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>三、板载触摸屏 (XPT2046) — 模拟SPI已改到PD口，释放PC8-PC12</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>模拟SPI</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>PD3</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>TP-CLK</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>触摸屏SPI时钟</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>PC9</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>TP-CS</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>触摸SPI片选</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PC8→PD3</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>模拟SPI GPIO输出</t>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>低电平有效</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>PD4</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>TP-CS</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>触摸屏SPI片选</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>PC10</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>TP-MOSI</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>触摸SPI数据出</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PC9→PD4</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>低电平有效</t>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>模拟SPI</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>PD5</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>TP-MOSI</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>触摸屏SPI数据出</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>PC11</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>TP-MISO</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>触摸SPI数据入</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>模拟SPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>PC12</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>TP-PENIRQ</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>触摸中断</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>低电平=有触摸</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>四、板载SPI Flash (W25Q64) — 硬件SPI1，不动</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>PA4</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>FLASH-CS</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>W25Q64片选</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PC10→PD5</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>模拟SPI</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>PD6</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>TP-MISO</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>触摸屏SPI数据入</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PC11→PD6</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>模拟SPI</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>PD7</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>TP-PENIRQ</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>触摸屏中断/按下检测</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PC12→PD7</t>
-        </is>
-      </c>
-      <c r="G25" s="13" t="inlineStr">
-        <is>
-          <t>低电平=有触摸</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>四、板载SPI Flash (W25Q64) — 硬件SPI1</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="11" t="n"/>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="11" t="n"/>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>SPI1 NSS</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
@@ -1401,17 +1401,17 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>PA4</t>
+          <t>PA5</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>FLASH-CS</t>
+          <t>FLASH-SCK</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>W25Q64片选</t>
+          <t>W25Q64时钟</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -1421,12 +1421,12 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>硬件SPI1 NSS</t>
+          <t>SPI1 SCK</t>
         </is>
       </c>
     </row>
@@ -1438,32 +1438,32 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>PA5</t>
+          <t>PA6</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>FLASH-SCK</t>
+          <t>FLASH-MISO</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>W25Q64时钟</t>
+          <t>W25Q64数据入</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>硬件SPI1 SCK</t>
+          <t>SPI1 MISO</t>
         </is>
       </c>
     </row>
@@ -1475,134 +1475,134 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>PA6</t>
+          <t>PA7</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>FLASH-MISO</t>
+          <t>FLASH-MOSI</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>W25Q64数据入</t>
+          <t>W25Q64数据出</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>硬件SPI1 MISO</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+          <t>SPI1 MOSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>五、板载蜂鸣器 — 不动</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>PA7</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>FLASH-MOSI</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>W25Q64数据出</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>PC1</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>BEEP</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>有源蜂鸣器</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>硬件SPI1 MOSI</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>五、板载蜂鸣器</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>跳帽J7 BEEP&lt;-&gt;C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>六、板载CH340调试串口 — USART1，不动</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>PC1</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>BEEP</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>有源蜂鸣器</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>PA9</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>CH340-TXD</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>CH340 RXD(MCU发)</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>✅ 跳帽J7选BEEP&lt;-&gt;C1</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>不接电位器，不能同时接VAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>六、UWB基站 (GC-P2304-GS-2) — USART2</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>USART1_TX，调试输出</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
@@ -1612,319 +1612,319 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>PA2</t>
+          <t>PA10</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>UWB-TXD</t>
+          <t>CH340-RXD</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>基站RXD(MCU发)</t>
+          <t>CH340 TXD(MCU收)</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>✅ 无冲突 — USART2_TX</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>115200,8N1</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>PA3</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>UWB-RXD</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>基站TXD(MCU收)</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>✅ 无冲突 — USART2_RX</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>测距/角度数据</t>
-        </is>
-      </c>
+          <t>USART1_RX，接收指令</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>七、UWB基站 (GC-P2304-GS-2) — USART2，不动</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>3.3V</t>
+          <t>PA2</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>UWB-VCC</t>
+          <t>UWB-TXD</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>基站电源</t>
+          <t>基站RXD(MCU发)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
+          <t>✅ 保持原样不动</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>2.0~3.6V</t>
+          <t>USART2_TX，115200</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>PA3</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>UWB-RXD</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>基站TXD(MCU收)</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>✅ 保持原样不动</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>USART2_RX，测距数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>UWB-VCC</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>基站电源</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>✅ 无冲突</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>2.0~3.6V</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>GND</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr">
         <is>
           <t>UWB-GND</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D39" s="9" t="inlineStr">
         <is>
           <t>基站地</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>GND</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>✅ 无冲突</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>共地</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>七、DL-20无线串口 — UART4(PC10/PC11)，不再占用USART1</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="n"/>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="11" t="n"/>
-      <c r="E38" s="11" t="n"/>
-      <c r="F38" s="11" t="n"/>
-      <c r="G38" s="11" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>PC10</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>八、DL-20无线串口 — 软件串口(PA0/PA1)，不占任何硬件USART</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>PA0</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>DL-TXD</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>DL-20 RXD(MCU发)</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E41" s="13" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PA9(USART1)→UART4_TX(PC10)</t>
-        </is>
-      </c>
-      <c r="G39" s="13" t="inlineStr">
-        <is>
-          <t>PC10原触摸屏MOSI，已改到PD5</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="12" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>PC11</t>
-        </is>
-      </c>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>🔧 软件串口TX — 所有硬件USART已被占用</t>
+        </is>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>用Timer定时翻转GPIO模拟9600波特率</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>PA1</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>DL-RXD</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D42" s="13" t="inlineStr">
         <is>
           <t>DL-20 TXD(MCU收)</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E42" s="13" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PA10(USART1)→UART4_RX(PC11)</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="inlineStr">
-        <is>
-          <t>PC11原触摸屏MISO，已改到PD6</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>🔧 软件串口RX — 取下J7 TPAD跳帽</t>
+        </is>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>用外部中断+定时器采样9600波特率</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>3.3V</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C43" s="9" t="inlineStr">
         <is>
           <t>DL-VCC</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D43" s="9" t="inlineStr">
         <is>
           <t>DL-20电源</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E43" s="9" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>✅ 无冲突</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G43" s="9" t="inlineStr">
         <is>
           <t>2.8~5.5V</t>
         </is>
       </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>DL-GND</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>DL-20地</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>共地</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>八、板载CH340调试串口 — USART1(PA9/PA10)，独立运行，不与DL-20争用</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n"/>
-      <c r="C43" s="5" t="n"/>
-      <c r="D43" s="5" t="n"/>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
@@ -1934,84 +1934,84 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>PA9</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>CH340-TXD</t>
+          <t>DL-GND</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>CH340 RXD(MCU发)</t>
+          <t>DL-20地</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>✅ 独立调试，不接DL-20</t>
+          <t>✅ 无冲突</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>USART1_TX，调试输出</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
+          <t>共地</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>九、4位拨码开关 — 用空闲IO，无冲突</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>PA10</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>CH340-RXD</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>CH340 TXD(MCU收)</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>PC0</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>SW1(ID3/MSB)</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>拨码开关位3</t>
+        </is>
+      </c>
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>✅ 独立调试，不接DL-20</t>
-        </is>
-      </c>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>USART1_RX，接收指令</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t>九、拨码开关(4位ID) — 改用PD口，避开所有冲突</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="n"/>
-      <c r="C46" s="11" t="n"/>
-      <c r="D46" s="11" t="n"/>
-      <c r="E46" s="11" t="n"/>
-      <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
+      <c r="F46" s="13" t="inlineStr">
+        <is>
+          <t>🔧 用空闲PC0</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>上拉输入，GND=0</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="12" t="inlineStr">
@@ -2021,17 +2021,17 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>PD8</t>
+          <t>PC2</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>SW1(ID3/MSB)</t>
+          <t>SW2(ID2)</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>拨码开关位3</t>
+          <t>拨码开关位2</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>🔧 已改 — 原PA0→PD8</t>
+          <t>🔧 用空闲PC2</t>
         </is>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>上拉输入，GND=0</t>
+          <t>上拉输入</t>
         </is>
       </c>
     </row>
@@ -2058,17 +2058,17 @@
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>PD9</t>
+          <t>PC3</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>SW2(ID2)</t>
+          <t>SW3(ID1)</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>拨码开关位2</t>
+          <t>拨码开关位1</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>🔧 已改 — 原PA1→PD9</t>
+          <t>🔧 用空闲PC3</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
@@ -2095,17 +2095,17 @@
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>PD10</t>
+          <t>PA8</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>SW3(ID1)</t>
+          <t>SW4(ID0/LSB)</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>拨码开关位1</t>
+          <t>拨码开关位0</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>🔧 已改 — 原PC0→PD10</t>
+          <t>🔧 用空闲PA8</t>
         </is>
       </c>
       <c r="G49" s="13" t="inlineStr">
@@ -2124,142 +2124,134 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="12" t="inlineStr">
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>十、状态指示LED — 外接，不碰板载LED(LCD占用)</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="11" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="11" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>PD11</t>
-        </is>
-      </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>SW4(ID0/LSB)</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>拨码开关位0</t>
-        </is>
-      </c>
-      <c r="E50" s="13" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 原PC13→PD11</t>
-        </is>
-      </c>
-      <c r="G50" s="13" t="inlineStr">
-        <is>
-          <t>上拉输入</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>十、状态指示LED — 外接，不占用LCD数据线</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="12" t="inlineStr">
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>PA15</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>LED-STATUS</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>外接状态LED</t>
+        </is>
+      </c>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="F51" s="13" t="inlineStr">
+        <is>
+          <t>🔧 用PA15(需禁用JTAG)</t>
+        </is>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>代码已禁用JTAG用SWD，PA15可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>十一、预留可用IO（LQFP64仅剩这些）</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="n"/>
+      <c r="C52" s="11" t="n"/>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="11" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>PC0</t>
-        </is>
-      </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>LED-GREEN</t>
-        </is>
-      </c>
-      <c r="D52" s="13" t="inlineStr">
-        <is>
-          <t>外接绿色LED</t>
-        </is>
-      </c>
-      <c r="E52" s="13" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F52" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 放弃PB0/PB1/PB5改用PC0</t>
-        </is>
-      </c>
-      <c r="G52" s="13" t="inlineStr">
-        <is>
-          <t>PC0原拨码开关，已改到PD10</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>PD0</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>预留(晶振)</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>8MHz晶振OSC_IN</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>❌ 接晶振尽量不用</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>PC13</t>
-        </is>
-      </c>
-      <c r="C53" s="13" t="inlineStr">
-        <is>
-          <t>LED-RED</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="inlineStr">
-        <is>
-          <t>外接红色LED</t>
-        </is>
-      </c>
-      <c r="E53" s="13" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F53" s="13" t="inlineStr">
-        <is>
-          <t>🔧 已改 — 放弃PB0/PB1/PB5改用PC13</t>
-        </is>
-      </c>
-      <c r="G53" s="13" t="inlineStr">
-        <is>
-          <t>注意PC13接RTC晶振，影响不大</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>十一、预留可用IO</t>
-        </is>
-      </c>
-      <c r="B54" s="11" t="n"/>
-      <c r="C54" s="11" t="n"/>
-      <c r="D54" s="11" t="n"/>
-      <c r="E54" s="11" t="n"/>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="11" t="n"/>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>PD1</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>预留(晶振)</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>8MHz晶振OSC_OUT</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>❌ 接晶振尽量不用</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="8" t="inlineStr">
@@ -2269,7 +2261,7 @@
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>PA0</t>
+          <t>PC13</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
@@ -2289,10 +2281,14 @@
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>✅ 空闲 — 原拨码开关已改到PD8</t>
-        </is>
-      </c>
-      <c r="G55" s="9" t="inlineStr"/>
+          <t>✅ 空闲但接RTC晶振</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>影响RTC，尽量不用</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
@@ -2302,7 +2298,7 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>PA1</t>
+          <t>PC14</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
@@ -2322,12 +2318,12 @@
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>✅ 空闲 — 注意TPAD跳帽J7</t>
+          <t>✅ 空闲但接RTC晶振</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>若需用PA1，取下TPAD跳帽</t>
+          <t>OSC32_OUT</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2335,7 @@
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>PA8</t>
+          <t>PC15</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
@@ -2359,351 +2355,30 @@
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>✅ 空闲</t>
+          <t>✅ 空闲但接RTC晶振</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>可做UWB RST</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>PA15</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr">
-        <is>
-          <t>预留IO4</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>✅ 空闲</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>JTAG_NJTRST</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B59" s="9" t="inlineStr">
-        <is>
-          <t>PC8</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>预留IO5</t>
-        </is>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="inlineStr">
-        <is>
-          <t>✅ 空闲 — 原触摸屏已释放</t>
-        </is>
-      </c>
-      <c r="G59" s="9" t="inlineStr"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="inlineStr">
-        <is>
-          <t>PC9</t>
-        </is>
-      </c>
-      <c r="C60" s="7" t="inlineStr">
-        <is>
-          <t>预留IO6</t>
-        </is>
-      </c>
-      <c r="D60" s="7" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F60" s="7" t="inlineStr">
-        <is>
-          <t>✅ 空闲 — 原触摸屏已释放</t>
-        </is>
-      </c>
-      <c r="G60" s="7" t="inlineStr"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>PC12</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>预留IO7</t>
-        </is>
-      </c>
-      <c r="D61" s="9" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>✅ 空闲 — 原触摸屏PENIRQ已释放</t>
-        </is>
-      </c>
-      <c r="G61" s="9" t="inlineStr"/>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>PC14</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>预留IO8</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F62" s="7" t="inlineStr">
-        <is>
-          <t>✅ 空闲</t>
-        </is>
-      </c>
-      <c r="G62" s="7" t="inlineStr">
-        <is>
-          <t>OSC32_OUT，尽量不用</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="B63" s="9" t="inlineStr">
-        <is>
-          <t>PC15</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>预留IO9</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr">
-        <is>
-          <t>✅ 空闲</t>
-        </is>
-      </c>
-      <c r="G63" s="9" t="inlineStr">
-        <is>
-          <t>OSC32_IN，尽量不用</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>PD0</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>预留IO10</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F64" s="7" t="inlineStr">
-        <is>
-          <t>✅ 空闲</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
-        <is>
-          <t>接8MHz晶振，尽量不用</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>PD1</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>预留IO11</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E65" s="9" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="inlineStr">
-        <is>
-          <t>✅ 空闲</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>接8MHz晶振，尽量不用</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>PD12~PD15</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>预留IO12~15</t>
-        </is>
-      </c>
-      <c r="D66" s="7" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F66" s="7" t="inlineStr">
-        <is>
-          <t>✅ 空闲</t>
-        </is>
-      </c>
-      <c r="G66" s="7" t="inlineStr">
-        <is>
-          <t>大量PD口可用</t>
+          <t>OSC32_IN</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A45:G45"/>
     <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2715,7 +2390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2736,7 +2411,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>芯片: STM32F103RCT6 (LQFP64) | 不接LCD/触摸屏 → GPIOB/C/D全部空闲 | 外接UWB标签+DL-20+按键+LED+WiFi预留</t>
+          <t>STM32F103RCT6 LQFP64 | 不接LCD/触摸屏 → GPIOB/C/D大量空闲 | 全部用硬件USART</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2573,7 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>BOOT0引脚</t>
+          <t>BOOT0</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -2930,7 +2605,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>SWD调试接口</t>
+          <t>SWD调试</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -2962,7 +2637,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>SWD调试接口</t>
+          <t>SWD调试</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2979,7 +2654,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>二、无线串口 (DL-20) — USART1，独占PA9/PA10</t>
+          <t>二、无线串口 (DL-20) — USART1，独占</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
@@ -3411,7 +3086,7 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>六、WiFi预留 (ESP8266/ESP32-C3) — USART3</t>
+          <t>六、WiFi预留 (ESP8266) — USART3</t>
         </is>
       </c>
       <c r="B28" s="11" t="n"/>
@@ -3512,7 +3187,7 @@
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>无冲突 — 注意峰值电流&gt;500mA</t>
+          <t>无冲突 — 峰值&gt;500mA</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3455,7 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>空闲 — JTAG_NJTRST</t>
+          <t>空闲 — 需禁用JTAG</t>
         </is>
       </c>
     </row>
@@ -3941,38 +3616,6 @@
       <c r="F45" s="9" t="inlineStr">
         <is>
           <t>PD0/PD1接晶振，PD2自由</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>PD3~PD15</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>预留IO38~50</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>全部空闲</t>
         </is>
       </c>
     </row>
@@ -3998,16 +3641,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4045,7 +3688,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>所用USART</t>
+          <t>所用串口</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -4057,7 +3700,8 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>GC-P2304-GS-2 (UWB基站)</t>
+          <t>GC-P2304-GS-2
+(UWB基站)</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -4202,7 +3846,8 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>GTM1000 (UWB标签)</t>
+          <t>GTM1000
+(UWB标签)</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -4324,7 +3969,7 @@
           <t>GND</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4357,7 +4002,7 @@
           <t>PB0</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4380,7 +4025,8 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>DL-20 (无线串口)</t>
+          <t>DL-20
+(无线串口)</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -4395,7 +4041,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>→ PC11(UART4_RX)</t>
+          <t>→ PA1(软件串口RX)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -4403,9 +4049,9 @@
           <t>→ PA10(USART1_RX)</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>门锁UART4/钥匙USART1</t>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>门锁软件串口/钥匙USART1</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -4428,7 +4074,7 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>← PC10(UART4_TX)</t>
+          <t>← PA0(软件串口TX)</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -4436,9 +4082,9 @@
           <t>← PA9(USART1_TX)</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>门锁UART4/钥匙USART1</t>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>门锁软件串口/钥匙USART1</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -4525,7 +4171,8 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>ESP8266 (WiFi预留)</t>
+          <t>ESP8266
+(WiFi预留)</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -4685,7 +4332,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>PD8</t>
+          <t>PC0</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -4718,7 +4365,7 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>PD9</t>
+          <t>PC2</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -4751,7 +4398,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>PD10</t>
+          <t>PC3</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -4784,7 +4431,7 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>PD11</t>
+          <t>PA8</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -4820,86 +4467,28 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>STATUS</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>绿色LED</t>
+          <t>状态LED</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>PC0</t>
+          <t>PA15</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PB5</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr"/>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>替代原PB0</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="16" t="n"/>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>红色LED</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>PC13</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr"/>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>替代原PB5</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="17" t="n"/>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>STATUS</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>状态LED</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>PB5</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr"/>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>钥匙端只有一个状态LED</t>
+          <t>门锁PA15/钥匙PB5</t>
         </is>
       </c>
     </row>
@@ -4907,10 +4496,10 @@
   <mergeCells count="12">
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A30:A32"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A30"/>
     <mergeCell ref="A20:A23"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A29:G29"/>
@@ -4928,7 +4517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4942,7 +4531,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>引脚冲突解决对照表（旧方案 → 新方案）</t>
+          <t>引脚冲突解决对照表（屏幕不动方案）</t>
         </is>
       </c>
     </row>
@@ -4986,7 +4575,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>PB0~PB15 = LCD数据总线 vs 板载LED(PB0/PB1/PB5)</t>
+          <t>PB0~PB15 = LCD数据总线 vs 板载LED</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -5001,12 +4590,12 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>放弃板载LED，外接LED到PC0/PC13</t>
+          <t>放弃板载LED，外接LED到PA15</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>LCD是必须功能，LED改为外接</t>
+          <t>LCD必须用，LED改外接</t>
         </is>
       </c>
     </row>
@@ -5028,17 +4617,17 @@
       </c>
       <c r="D5" s="20" t="inlineStr">
         <is>
-          <t>DL-20和CH340都接USART1(PA9/PA10) → 冲突</t>
+          <t>DL-20和CH340都接USART1 → 冲突</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>DL-20改到UART4(PC10/PC11)，CH340独占USART1</t>
+          <t>DL-20改用软件串口(PA0/PA1)，CH340独占USART1</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>UART4释放后可用(触摸屏已改到PD)</t>
+          <t>所有硬件USART已被占满，DL-20用软件串口9600</t>
         </is>
       </c>
     </row>
@@ -5050,7 +4639,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>PC8~PC12 = 触摸屏(模拟SPI) vs UART4(PC10/PC11)</t>
+          <t>PA0/PA1 = 拨码开关 vs 电容按键(TPAD)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -5060,17 +4649,17 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>触摸屏占PC8~PC12，但UART4需要PC10/PC11 → 冲突</t>
+          <t>拨码开关用PA0/PA1，PA1有TPAD跳帽 → 冲突</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>触摸屏模拟SPI改到PD3~PD7，释放PC8~PC12</t>
+          <t>拨码开关改到PC0/PC2/PC3/PA8，PA0/PA1给DL-20软件串口</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>触摸屏是软件模拟SPI，任意GPIO均可</t>
+          <t>PC0/PC2/PC3/PA8全部空闲</t>
         </is>
       </c>
     </row>
@@ -5082,7 +4671,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>PA0/PA1 = 拨码开关 vs 电容按键(PA1有TPAD跳帽)</t>
+          <t>PC13 = 拨码开关 vs RTC晶振</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -5092,17 +4681,17 @@
       </c>
       <c r="D7" s="20" t="inlineStr">
         <is>
-          <t>拨码开关用PA0/PA1，但PA1有TPAD跳帽冲突</t>
+          <t>拨码开关用PC13，但PC13接RTC晶振</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>拨码开关改到PD8~PD11</t>
+          <t>拨码开关不用PC13，改用PA8</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>PD口大量空闲</t>
+          <t>PC13保留给RTC</t>
         </is>
       </c>
     </row>
@@ -5114,7 +4703,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>PC13 = 拨码开关 vs RTC晶振(32.768kHz)</t>
+          <t>PC8~PC12 = 触摸屏 vs UART4/UART5</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -5124,17 +4713,17 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>拨码开关用PC13，但PC13接RTC晶振</t>
+          <t>触摸屏占PC8~PC12，UART4(PC10/11)/UART5(PC12)冲突</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>拨码开关改到PD11，PC13释放</t>
+          <t>触摸屏不动，DL-20改软件串口不占UART</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>PC13影响RTC，最好不用</t>
+          <t>屏幕接线完全不动</t>
         </is>
       </c>
     </row>
@@ -5146,27 +4735,27 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>PC0 = 拨码开关 vs 蜂鸣器/电位器(PC1跳帽复用)</t>
+          <t>PB0~PB15 = 钥匙端误标冲突</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>门锁端</t>
+          <t>钥匙端</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>拨码开关用PC0，PC0有跳帽复用</t>
+          <t>旧表标注"注意冲突"但钥匙端无LCD</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>拨码开关改到PD10，PC0改做外接LED</t>
+          <t>标注"无冲突"，PB0/PB1/PB5正常用</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>PC0释放后可做其他用途</t>
+          <t>钥匙端不接LCD</t>
         </is>
       </c>
     </row>
@@ -5178,7 +4767,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>PB0~PB15 = 误标"冲突"但实际无冲突</t>
+          <t>PA9/PA10 = 钥匙端误标分时复用</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -5188,17 +4777,17 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>旧表标注"注意冲突"，但钥匙端无LCD</t>
+          <t>旧表标注分时复用，但钥匙端无CH340</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>直接标注"无冲突"，PB0/PB1/PB5正常使用</t>
+          <t>标注"无冲突"，DL-20独占USART1</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>钥匙端不接LCD，GPIOB全部空闲</t>
+          <t>钥匙端不需要CH340</t>
         </is>
       </c>
     </row>
@@ -5210,59 +4799,27 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>PA9/PA10 = 误标"分时复用"但钥匙端无CH340</t>
+          <t>LQFP64封装PD口限制</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>钥匙端</t>
+          <t>两端</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>旧表标注分时复用，但钥匙端无CH340</t>
+          <t>之前方案用PD3~PD15，但LQFP64只有PD0/PD1/PD2</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>直接标注"无冲突"，DL-20独占USART1</t>
+          <t>全部改用PA/PC口，不依赖PD3~PD15</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>钥匙端不需要CH340调试</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>PC1 = 蜂鸣器 vs 电位器(跳帽选择)</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>门锁端</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>蜂鸣器和电位器都接PC1，通过跳帽选择</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>保持跳帽选择：J7 BEEP&lt;-&gt;C1接蜂鸣器</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>同一时间只能选一个功能</t>
+          <t>LQFP64仅51个GPIO</t>
         </is>
       </c>
     </row>
@@ -5315,12 +4872,12 @@
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>触摸屏引脚变更</t>
+          <t>软件串口实现</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>XPT2046触摸屏模拟SPI从PC8~PC12改到PD3~PD7(CLK/CS/MOSI/MISO/PENIRQ)。需要修改`bsp_xpt2046_lcd.h`中的引脚定义，重新编译。</t>
+          <t>门锁端DL-20用软件串口(PA0 TX / PA1 RX)，波特率9600。TX用Timer定时翻转GPIO，RX用外部中断下降沿触发+定时器采样。72MHz下9600波特率软件串口非常稳定。</t>
         </is>
       </c>
       <c r="C4" s="21" t="inlineStr">
@@ -5332,12 +4889,12 @@
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>DL-20端口变更</t>
+          <t>屏幕接线不变</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>门锁端DL-20从USART1(PA9/PA10)改到UART4(PC10/PC11)。需要新增UART4初始化代码，参考现有USART驱动。</t>
+          <t>LCD(ILI9341)和触摸屏(XPT2046)的接线完全保持原样，不需要修改任何现有驱动代码。PB0~PB15、PC4~PC7、PC8~PC12、PD2全部不动。</t>
         </is>
       </c>
       <c r="C5" s="22" t="inlineStr">
@@ -5349,12 +4906,12 @@
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>拨码开关引脚变更</t>
+          <t>USART资源分配</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>门锁端4位拨码开关从PA0/PA1/PC0/PC13改到PD8/PD9/PD10/PD11。需要修改读取ID的代码。</t>
+          <t>门锁端：USART1(CH340调试) + USART2(UWB基站) + 软件串口(DL-20)。钥匙端：USART1(DL-20) + USART2(UWB标签) + USART3(WiFi预留)。</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
@@ -5366,12 +4923,12 @@
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>LED方案变更</t>
+          <t>拨码开关引脚</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>门锁端放弃板载LED(PB0/PB1/PB5与LCD冲突)，改用外接LED接到PC0(绿)和PC13(红)。钥匙端保持PB5做状态LED。</t>
+          <t>门锁端4位拨码开关用PC0/PC2/PC3/PA8，全部是空闲引脚，无任何冲突。上拉输入，接GND=0，悬空=1。</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -5383,46 +4940,46 @@
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>USART资源分配</t>
+          <t>LED方案</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>门锁端：USART1(CH340调试) + USART2(UWB基站) + UART4(DL-20)。钥匙端：USART1(DL-20) + USART2(UWB标签) + USART3(WiFi预留)。</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>门锁端放弃板载LED(PB0/PB1/PB5与LCD冲突)，外接LED到PA15。需确保代码禁用JTAG(AFIO_Remap_SWJ_JTAGDisable)以释放PA15。钥匙端用PB5。</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>电源设计</t>
+          <t>LQFP64封装限制</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>门锁端USB 5V供电，板载AMS1117-3.3。钥匙端3.7V锂电池+AMS1117-3.3 LDO。</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>STM32F103RCT6 LQFP64仅有PD0/PD1/PD2三个PD引脚，PD3~PD15不存在。所有外接功能必须用PA/PC口。</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>WiFi模块</t>
+          <t>电源设计</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>ESP8266/ESP32-C3峰值电流&gt;500mA，钥匙端启用WiFi时需注意电池容量。</t>
+          <t>门锁端USB 5V供电，板载AMS1117-3.3。钥匙端3.7V锂电池+AMS1117-3.3 LDO。</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -5473,7 +5030,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>门锁端和钥匙端DL-20需设置为相同信道(默认信道1)，建议点对点模式。</t>
+          <t>门锁端和钥匙端DL-20需设置为相同信道(默认信道1)，建议点对点模式。门锁端波特率建议设9600(配合软件串口)。</t>
         </is>
       </c>
       <c r="C13" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Switch from LCD to OLED (SSD1306 I2C) - massive pin savings
OLED only needs PB6/PB7 (I2C1), freeing entire GPIOB

Key changes:

- OLED: PB6(SCL)/PB7(SDA) I2C, 4.7k pull-ups required

- Onboard LEDs (PB0/PB1/PB5) now usable (no LCD conflict)

- DL-20 moved to USART3 PB10/PB11 (hardware serial, 115200)

- DIP switch: PA0/PC0/PC2/PC3

- Key input: PA1(OK), PA8(CANCEL) - OLED has no touch

- All hardware USARTs used, no software serial needed

- Touchscreen removed (OLED not compatible)

- Added LCD vs OLED comparison sheet
</commit_message>
<xml_diff>
--- a/Doc/硬件引脚分配表.xlsx
+++ b/Doc/硬件引脚分配表.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="智能门锁端接线" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数字钥匙端接线" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模块接线速查" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="冲突解决对照表" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更说明" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计说明" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
@@ -212,11 +212,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -235,16 +232,19 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -620,21 +620,20 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>野火STM32F103_MINI 智能门锁端 硬件接线表（屏幕不动，无冲突）</t>
+          <t>野火STM32F103_MINI 智能门锁端 硬件接线表（OLED方案）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>STM32F103RCT6 LQFP64(仅PD0/PD1/PD2) | LCD+触摸屏接线完全不动 | DL-20用软件串口 | 所有硬件USART不冲突</t>
+          <t>放弃LCD → OLED(I2C: PB6/PB7) | 释放GPIOB全部引脚 | 板载LED恢复使用 | 全部硬件USART无冲突</t>
         </is>
       </c>
     </row>
@@ -665,11 +664,6 @@
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>冲突解决</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -686,7 +680,6 @@
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -716,12 +709,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>板载，无冲突</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>USB 5V输入</t>
+          <t>板载，USB 5V输入</t>
         </is>
       </c>
     </row>
@@ -753,11 +741,6 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>板载，无冲突</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
           <t>所有模块共地</t>
         </is>
       </c>
@@ -790,11 +773,6 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>板载，无冲突</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
           <t>低电平复位</t>
         </is>
       </c>
@@ -827,11 +805,6 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>板载，无冲突</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
           <t>接GND正常，接VCC串口下载</t>
         </is>
       </c>
@@ -864,11 +837,6 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>板载，无冲突</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
           <t>接DAP/J-Link</t>
         </is>
       </c>
@@ -901,11 +869,6 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>板载，无冲突</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
           <t>接DAP/J-Link</t>
         </is>
       </c>
@@ -913,7 +876,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>二、板载LCD (ILI9341) — 接线完全不动</t>
+          <t>二、OLED显示屏 (SSD1306/SH1106 I2C)</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
@@ -921,7 +884,6 @@
       <c r="D12" s="11" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -931,17 +893,17 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>PB0~PB15</t>
+          <t>PB6</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>LCD-D0~D15</t>
+          <t>OLED-SCL</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>LCD 16位数据</t>
+          <t>OLED I2C时钟</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -951,12 +913,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>8080并口，占整个GPIOB</t>
+          <t>I2C1_SCL，需上拉电阻4.7k</t>
         </is>
       </c>
     </row>
@@ -968,32 +925,27 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>PB7</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>LCD-CS</t>
+          <t>OLED-SDA</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>LCD片选</t>
+          <t>OLED I2C数据</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>IO</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>低电平有效</t>
+          <t>I2C1_SDA，需上拉电阻4.7k</t>
         </is>
       </c>
     </row>
@@ -1005,32 +957,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>PC5</t>
+          <t>3.3V</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>LCD-RD</t>
+          <t>OLED-VCC</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>LCD读使能</t>
+          <t>OLED电源</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>低电平有效</t>
+          <t>3.3V供电</t>
         </is>
       </c>
     </row>
@@ -1042,121 +989,105 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>PC6</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>LCD-WR</t>
+          <t>OLED-GND</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>LCD写使能</t>
+          <t>OLED地</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>低电平有效</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>PC7</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>LCD-DC</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>LCD数据/命令</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>0=命令,1=数据</t>
-        </is>
-      </c>
+          <t>共地</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>三、板载LED（GPIOB释放后恢复使用）</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>PB0</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>LED-G</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>绿色LED</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>板载绿色LED，无冲突</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>PD2</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>LCD-BL</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>LCD背光</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>PB1</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>LED-B</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>蓝色LED</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>高电平点亮</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>三、板载触摸屏 (XPT2046) — 接线完全不动</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>板载蓝色LED，无冲突</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1166,17 +1097,17 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>PC8</t>
+          <t>PB5</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>TP-CLK</t>
+          <t>LED-R</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>触摸SPI时钟</t>
+          <t>红色LED</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -1184,73 +1115,43 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>模拟SPI</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>PC9</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>TP-CS</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>触摸SPI片选</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>低电平有效</t>
-        </is>
-      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>板载红色LED，无冲突</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>四、板载SPI Flash (W25Q64) — 硬件SPI1</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>PC10</t>
+          <t>PA4</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>TP-MOSI</t>
+          <t>FLASH-CS</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>触摸SPI数据出</t>
+          <t>W25Q64片选</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -1260,158 +1161,137 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>模拟SPI</t>
+          <t>SPI1 NSS</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>PC11</t>
+          <t>PA5</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>TP-MISO</t>
+          <t>FLASH-SCK</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>触摸SPI数据入</t>
+          <t>W25Q64时钟</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>模拟SPI</t>
+          <t>SPI1 SCK</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>PA6</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>FLASH-MISO</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>W25Q64数据入</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>SPI1 MISO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>PC12</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>TP-PENIRQ</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>触摸中断</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>低电平=有触摸</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>四、板载SPI Flash (W25Q64) — 硬件SPI1，不动</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>PA4</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>FLASH-CS</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>W25Q64片选</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>PA7</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>FLASH-MOSI</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>W25Q64数据出</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>SPI1 NSS</t>
-        </is>
-      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>SPI1 MOSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>五、板载蜂鸣器</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>PA5</t>
+          <t>PC1</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>FLASH-SCK</t>
+          <t>BEEP</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>W25Q64时钟</t>
+          <t>有源蜂鸣器</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -1421,771 +1301,689 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>SPI1 SCK</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>PA6</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>FLASH-MISO</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>W25Q64数据入</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>SPI1 MISO</t>
-        </is>
-      </c>
+          <t>跳帽J7 BEEP&lt;-&gt;C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>六、板载CH340调试串口 — USART1</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>PA9</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>CH340-TXD</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>CH340 RXD(MCU发)</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>USART1_TX，调试输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>PA10</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>CH340-RXD</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>CH340 TXD(MCU收)</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>USART1_RX，接收指令</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>七、UWB基站 (GC-P2304-GS-2) — USART2</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>PA7</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>FLASH-MOSI</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>W25Q64数据出</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>PA2</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>UWB-TXD</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>基站RXD(MCU发)</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>SPI1 MOSI</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>五、板载蜂鸣器 — 不动</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="11" t="n"/>
-      <c r="F30" s="11" t="n"/>
-      <c r="G30" s="11" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>PC1</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>BEEP</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>有源蜂鸣器</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G31" s="9" t="inlineStr">
-        <is>
-          <t>跳帽J7 BEEP&lt;-&gt;C1</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>六、板载CH340调试串口 — USART1，不动</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="11" t="n"/>
-      <c r="G32" s="11" t="n"/>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>USART2_TX，115200</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>PA9</t>
+          <t>PA3</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>CH340-TXD</t>
+          <t>UWB-RXD</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>CH340 RXD(MCU发)</t>
+          <t>基站TXD(MCU收)</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>USART1_TX，调试输出</t>
+          <t>USART2_RX，测距数据</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>UWB-VCC</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>基站电源</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>2.0~3.6V</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>PA10</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>CH340-RXD</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>CH340 TXD(MCU收)</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>USART1_RX，接收指令</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>七、UWB基站 (GC-P2304-GS-2) — USART2，不动</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>PA2</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>UWB-TXD</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>基站RXD(MCU发)</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>USART2_TX，115200</t>
-        </is>
-      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>UWB-GND</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>基站地</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>共地</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>八、DL-20无线串口 — USART3(PB10/PB11)，独占</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>PA3</t>
+          <t>PB10</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>UWB-RXD</t>
+          <t>DL-TXD</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>基站TXD(MCU收)</t>
+          <t>DL-20 RXD(MCU发)</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>✅ 保持原样不动</t>
-        </is>
-      </c>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>USART2_RX，测距数据</t>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>USART3_TX，GPIOB释放后可用</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>3.3V</t>
+          <t>PB11</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>UWB-VCC</t>
+          <t>DL-RXD</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>基站电源</t>
+          <t>DL-20 TXD(MCU收)</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>PWR</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>2.0~3.6V</t>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>USART3_RX，GPIOB释放后可用</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>DL-VCC</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>DL-20电源</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>2.8~5.5V</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>GND</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>UWB-GND</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>基站地</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>DL-GND</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>DL-20地</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>GND</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>共地</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>八、DL-20无线串口 — 软件串口(PA0/PA1)，不占任何硬件USART</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="n"/>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="11" t="n"/>
-      <c r="E40" s="11" t="n"/>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>九、4位拨码开关（ID设置）</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>PA0</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>DL-TXD</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>DL-20 RXD(MCU发)</t>
-        </is>
-      </c>
-      <c r="E41" s="13" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F41" s="13" t="inlineStr">
-        <is>
-          <t>🔧 软件串口TX — 所有硬件USART已被占用</t>
-        </is>
-      </c>
-      <c r="G41" s="13" t="inlineStr">
-        <is>
-          <t>用Timer定时翻转GPIO模拟9600波特率</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>PA1</t>
-        </is>
-      </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>DL-RXD</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>DL-20 TXD(MCU收)</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>SW1(ID3/MSB)</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>拨码开关位3</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr">
-        <is>
-          <t>🔧 软件串口RX — 取下J7 TPAD跳帽</t>
-        </is>
-      </c>
-      <c r="G42" s="13" t="inlineStr">
-        <is>
-          <t>用外部中断+定时器采样9600波特率</t>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>上拉输入，GND=0</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>3.3V</t>
+          <t>PC0</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>DL-VCC</t>
+          <t>SW2(ID2)</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>DL-20电源</t>
+          <t>拨码开关位2</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>2.8~5.5V</t>
+          <t>上拉输入</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>SW3(ID1)</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>拨码开关位1</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>DL-GND</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>DL-20地</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>✅ 无冲突</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>共地</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>九、4位拨码开关 — 用空闲IO，无冲突</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="5" t="n"/>
-      <c r="G45" s="5" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="12" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>SW4(ID0/LSB)</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>拨码开关位0</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>十、按键输入（OLED无触摸，用按键交互）</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>PC0</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>SW1(ID3/MSB)</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>拨码开关位3</t>
-        </is>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>PA1</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>KEY-OK</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>确认按键</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F46" s="13" t="inlineStr">
-        <is>
-          <t>🔧 用空闲PC0</t>
-        </is>
-      </c>
-      <c r="G46" s="13" t="inlineStr">
-        <is>
-          <t>上拉输入，GND=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>上拉输入，取下J7 TPAD跳帽</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>PC2</t>
-        </is>
-      </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>SW2(ID2)</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>拨码开关位2</t>
-        </is>
-      </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>PA8</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>KEY-CANCEL</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>取消按键</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F47" s="13" t="inlineStr">
-        <is>
-          <t>🔧 用空闲PC2</t>
-        </is>
-      </c>
-      <c r="G47" s="13" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>上拉输入</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="12" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>十一、预留可用IO</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
-      <c r="C48" s="13" t="inlineStr">
-        <is>
-          <t>SW3(ID1)</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
-        <is>
-          <t>拨码开关位1</t>
-        </is>
-      </c>
-      <c r="E48" s="13" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="inlineStr">
-        <is>
-          <t>🔧 用空闲PC3</t>
-        </is>
-      </c>
-      <c r="G48" s="13" t="inlineStr">
-        <is>
-          <t>上拉输入</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>PB2~PB4</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>预留IO1~3</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>IO</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="inlineStr">
+        <is>
+          <t>空闲</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>PA8</t>
-        </is>
-      </c>
-      <c r="C49" s="13" t="inlineStr">
-        <is>
-          <t>SW4(ID0/LSB)</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="inlineStr">
-        <is>
-          <t>拨码开关位0</t>
-        </is>
-      </c>
-      <c r="E49" s="13" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F49" s="13" t="inlineStr">
-        <is>
-          <t>🔧 用空闲PA8</t>
-        </is>
-      </c>
-      <c r="G49" s="13" t="inlineStr">
-        <is>
-          <t>上拉输入</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>十、状态指示LED — 外接，不碰板载LED(LCD占用)</t>
-        </is>
-      </c>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="11" t="n"/>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="11" t="n"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>PB8~PB9</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>预留IO4~5</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>IO</t>
+        </is>
+      </c>
+      <c r="F51" s="13" t="inlineStr">
+        <is>
+          <t>空闲</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>PA15</t>
-        </is>
-      </c>
-      <c r="C51" s="13" t="inlineStr">
-        <is>
-          <t>LED-STATUS</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="inlineStr">
-        <is>
-          <t>外接状态LED</t>
-        </is>
-      </c>
-      <c r="E51" s="13" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="F51" s="13" t="inlineStr">
-        <is>
-          <t>🔧 用PA15(需禁用JTAG)</t>
-        </is>
-      </c>
-      <c r="G51" s="13" t="inlineStr">
-        <is>
-          <t>代码已禁用JTAG用SWD，PA15可用</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="10" t="inlineStr">
-        <is>
-          <t>十一、预留可用IO（LQFP64仅剩这些）</t>
-        </is>
-      </c>
-      <c r="B52" s="11" t="n"/>
-      <c r="C52" s="11" t="n"/>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
-      <c r="G52" s="11" t="n"/>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>PB12~PB15</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>预留IO6~9</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>IO</t>
+        </is>
+      </c>
+      <c r="F52" s="13" t="inlineStr">
+        <is>
+          <t>空闲</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="8" t="inlineStr">
@@ -2195,30 +1993,29 @@
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>PD0</t>
+          <t>PC4~PC7</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>预留(晶振)</t>
+          <t>预留IO10~13</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>8MHz晶振OSC_IN</t>
+          <t>GPIO</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>❌ 接晶振尽量不用</t>
-        </is>
-      </c>
-      <c r="G53" s="9" t="inlineStr"/>
+          <t>IO</t>
+        </is>
+      </c>
+      <c r="F53" s="13" t="inlineStr">
+        <is>
+          <t>空闲（原LCD控制引脚）</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
@@ -2228,30 +2025,29 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>PD1</t>
+          <t>PC8~PC12</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>预留(晶振)</t>
+          <t>预留IO14~18</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>8MHz晶振OSC_OUT</t>
+          <t>GPIO</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>❌ 接晶振尽量不用</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr"/>
+          <t>IO</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="inlineStr">
+        <is>
+          <t>空闲（原触摸屏引脚）</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="8" t="inlineStr">
@@ -2261,12 +2057,12 @@
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>PC13</t>
+          <t>PC13~PC15</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>预留IO1</t>
+          <t>预留IO19~21</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2281,12 +2077,7 @@
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>✅ 空闲但接RTC晶振</t>
-        </is>
-      </c>
-      <c r="G55" s="9" t="inlineStr">
-        <is>
-          <t>影响RTC，尽量不用</t>
+          <t>接RTC晶振，尽量不用</t>
         </is>
       </c>
     </row>
@@ -2298,12 +2089,12 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>PC14</t>
+          <t>PD0~PD2</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>预留IO2</t>
+          <t>预留IO22~24</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -2318,67 +2109,25 @@
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>✅ 空闲但接RTC晶振</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>OSC32_OUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>PC15</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>预留IO3</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>IO</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>✅ 空闲但接RTC晶振</t>
-        </is>
-      </c>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>OSC32_IN</t>
+          <t>PD0/PD1接晶振，PD2自由</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2404,14 +2153,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>野火STM32F103_MINI 数字钥匙端 硬件接线表（无冲突）</t>
+          <t>野火STM32F103_MINI 数字钥匙端 硬件接线表</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>STM32F103RCT6 LQFP64 | 不接LCD/触摸屏 → GPIOB/C/D大量空闲 | 全部用硬件USART</t>
+          <t>不接LCD/OLED → GPIOB/C/D大量空闲 | 全部用硬件USART | 无冲突</t>
         </is>
       </c>
     </row>
@@ -2485,9 +2234,9 @@
           <t>PWR</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 建议3.7V锂电池+3.3V LDO</t>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>建议3.7V锂电池+3.3V LDO</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2266,7 @@
           <t>GND</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>无冲突</t>
         </is>
@@ -2549,7 +2298,7 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>无冲突</t>
         </is>
@@ -2581,9 +2330,9 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 接GND</t>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>接GND</t>
         </is>
       </c>
     </row>
@@ -2613,9 +2362,9 @@
           <t>IO</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 调试用</t>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>调试用</t>
         </is>
       </c>
     </row>
@@ -2645,16 +2394,16 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 调试用</t>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>调试用</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>二、无线串口 (DL-20) — USART1，独占</t>
+          <t>二、无线串口 (DL-20) — USART1</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
@@ -2689,9 +2438,9 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — USART1_TX，钥匙端无CH340</t>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>USART1_TX，钥匙端无CH340</t>
         </is>
       </c>
     </row>
@@ -2721,9 +2470,9 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — USART1_RX</t>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>USART1_RX</t>
         </is>
       </c>
     </row>
@@ -2753,9 +2502,9 @@
           <t>PWR</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 2.8~5.5V</t>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>2.8~5.5V</t>
         </is>
       </c>
     </row>
@@ -2785,9 +2534,9 @@
           <t>GND</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>无冲突</t>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>共地</t>
         </is>
       </c>
     </row>
@@ -2829,9 +2578,9 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — USART2_TX</t>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>USART2_TX</t>
         </is>
       </c>
     </row>
@@ -2861,9 +2610,9 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — USART2_RX</t>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>USART2_RX</t>
         </is>
       </c>
     </row>
@@ -2893,9 +2642,9 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 钥匙端无LCD，PB0空闲</t>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>5ms高电平脉冲唤醒</t>
         </is>
       </c>
     </row>
@@ -2925,9 +2674,9 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 钥匙端无LCD，PB1空闲</t>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>高电平使能</t>
         </is>
       </c>
     </row>
@@ -2957,9 +2706,9 @@
           <t>PWR</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 2.0~3.6V</t>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>2.0~3.6V</t>
         </is>
       </c>
     </row>
@@ -2989,9 +2738,9 @@
           <t>GND</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>无冲突</t>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>共地</t>
         </is>
       </c>
     </row>
@@ -3033,9 +2782,9 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 上拉输入</t>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
         </is>
       </c>
     </row>
@@ -3077,9 +2826,9 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 钥匙端无LCD，PB5空闲</t>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>钥匙端状态指示</t>
         </is>
       </c>
     </row>
@@ -3121,9 +2870,9 @@
           <t>OUT</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — USART3_TX，预留</t>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>USART3_TX，预留</t>
         </is>
       </c>
     </row>
@@ -3153,9 +2902,9 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — USART3_RX，预留</t>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>USART3_RX，预留</t>
         </is>
       </c>
     </row>
@@ -3185,9 +2934,9 @@
           <t>PWR</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>无冲突 — 峰值&gt;500mA</t>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>峰值电流&gt;500mA</t>
         </is>
       </c>
     </row>
@@ -3217,16 +2966,16 @@
           <t>GND</t>
         </is>
       </c>
-      <c r="F32" s="14" t="inlineStr">
-        <is>
-          <t>无冲突</t>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>共地</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>七、预留可用IO（钥匙端大量空闲）</t>
+          <t>七、预留可用IO</t>
         </is>
       </c>
       <c r="B33" s="5" t="n"/>
@@ -3455,7 +3204,7 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>空闲 — 需禁用JTAG</t>
+          <t>需禁用JTAG</t>
         </is>
       </c>
     </row>
@@ -3641,10 +3390,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
@@ -3698,25 +3447,25 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>GC-P2304-GS-2
-(UWB基站)</t>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>SSD1306
+OLED</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>TXD</t>
+          <t>SCL</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>串口发送</t>
+          <t>I2C时钟</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>→ PA3(USART2_RX)</t>
+          <t>PB6(I2C1_SCL)</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -3726,30 +3475,30 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>USART2</t>
+          <t>I2C1</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>基站→MCU，测距数据</t>
+          <t>需4.7k上拉</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="16" t="n"/>
+      <c r="A5" s="15" t="n"/>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>RXD</t>
+          <t>SDA</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>串口接收</t>
+          <t>I2C数据</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>← PA2(USART2_TX)</t>
+          <t>PB7(I2C1_SDA)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3759,17 +3508,17 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>USART2</t>
+          <t>I2C1</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>MCU→基站，AT指令</t>
+          <t>需4.7k上拉</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="16" t="n"/>
+      <c r="A6" s="15" t="n"/>
       <c r="B6" s="9" t="inlineStr">
         <is>
           <t>VCC</t>
@@ -3795,14 +3544,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>2.0~3.6V</t>
-        </is>
-      </c>
+      <c r="G6" s="9" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="17" t="n"/>
+      <c r="A7" s="16" t="n"/>
       <c r="B7" s="7" t="inlineStr">
         <is>
           <t>GND</t>
@@ -3828,14 +3573,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>共地</t>
-        </is>
-      </c>
+      <c r="G7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="8" customHeight="1">
-      <c r="A8" s="18" t="n"/>
+      <c r="A8" s="17" t="n"/>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
@@ -3844,15 +3585,15 @@
       <c r="G8" s="5" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>GTM1000
-(UWB标签)</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>GC-P2304-GS-2
+(UWB基站)</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>UART_TX</t>
+          <t>TXD</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -3862,14 +3603,14 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
+          <t>→ PA3(USART2_RX)</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>→ PA3(USART2_RX)</t>
-        </is>
-      </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
           <t>USART2</t>
@@ -3877,15 +3618,15 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>标签→MCU，透传数据</t>
+          <t>基站→MCU</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="16" t="n"/>
+      <c r="A10" s="15" t="n"/>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>UART_RX</t>
+          <t>RXD</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -3895,14 +3636,14 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
+          <t>← PA2(USART2_TX)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>← PA2(USART2_TX)</t>
-        </is>
-      </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
           <t>USART2</t>
@@ -3910,15 +3651,15 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>MCU→标签</t>
+          <t>MCU→基站</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="16" t="n"/>
+      <c r="A11" s="15" t="n"/>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>VDD</t>
+          <t>VCC</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -3928,12 +3669,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>3.3V</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -3961,206 +3702,206 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>共地</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1">
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>GTM1000
+(UWB标签)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>UART_TX</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>串口发送</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>→ PA3(USART2_RX)</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>USART2</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>标签→MCU</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>UART_RX</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>串口接收</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>← PA2(USART2_TX)</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>USART2</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>MCU→标签</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>VDD</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>电源</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>2.0~3.6V</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>GND</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>地</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>共地</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="17" t="n"/>
-      <c r="B13" s="7" t="inlineStr">
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>SOS</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>唤醒</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>PB0</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>5ms高电平脉冲</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="8" customHeight="1">
-      <c r="A14" s="18" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>DL-20
-(无线串口)</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>TXD</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>串口发送</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>→ PA1(软件串口RX)</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>→ PA10(USART1_RX)</t>
-        </is>
-      </c>
-      <c r="F15" s="14" t="inlineStr">
-        <is>
-          <t>门锁软件串口/钥匙USART1</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>DL-20发→MCU收</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>RXD</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>串口接收</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>← PA0(软件串口TX)</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>← PA9(USART1_TX)</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>门锁软件串口/钥匙USART1</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>MCU发→DL-20收</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="16" t="n"/>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>VCC</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>电源</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>3.3V</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>3.3V</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>2.8~5.5V</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="17" t="n"/>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>地</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>共地</t>
-        </is>
-      </c>
-    </row>
     <row r="19" ht="8" customHeight="1">
-      <c r="A19" s="19" t="n"/>
+      <c r="A19" s="18" t="n"/>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
       <c r="D19" s="11" t="n"/>
@@ -4169,10 +3910,10 @@
       <c r="G19" s="11" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>ESP8266
-(WiFi预留)</t>
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>DL-20
+(无线串口)</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -4187,118 +3928,118 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
+          <t>→ PB11(USART3_RX)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>→ PA10(USART1_RX)</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>门锁USART3/钥匙USART1</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>DL-20发→MCU收</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>RXD</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>串口接收</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>← PB10(USART3_TX)</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>← PA9(USART1_TX)</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>门锁USART3/钥匙USART1</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>MCU发→DL-20收</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>VCC</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>电源</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>→ PB11(USART3_RX)</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>USART3</t>
-        </is>
-      </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>WiFi→MCU</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="16" t="n"/>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>RXD</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>串口接收</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>2.8~5.5V</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="16" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>地</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>← PB10(USART3_TX)</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>USART3</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>MCU→WiFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="16" t="n"/>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>VCC</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>电源</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>3.3V</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>峰值&gt;500mA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="17" t="n"/>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>地</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
           <t>共地</t>
@@ -4306,7 +4047,7 @@
       </c>
     </row>
     <row r="24" ht="8" customHeight="1">
-      <c r="A24" s="18" t="n"/>
+      <c r="A24" s="17" t="n"/>
       <c r="B24" s="5" t="n"/>
       <c r="C24" s="5" t="n"/>
       <c r="D24" s="5" t="n"/>
@@ -4315,143 +4056,144 @@
       <c r="G24" s="5" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>4位拨码开关</t>
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>ESP8266
+(WiFi预留)</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>TXD</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>ID3(MSB)</t>
+          <t>串口发送</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>PC0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
+          <t>→ PB11(USART3_RX)</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>USART3</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>WiFi→MCU</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="15" t="n"/>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>RXD</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>串口接收</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>← PB10(USART3_TX)</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>USART3</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>MCU→WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="15" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>VCC</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>电源</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>上拉输入</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="16" t="n"/>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>SW2</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>ID2</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>PC2</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>3.3V</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>峰值&gt;500mA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="16" t="n"/>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>地</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>上拉输入</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="16" t="n"/>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>SW3</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>ID1</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>GND</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>上拉输入</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="17" t="n"/>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>SW4</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>ID0(LSB)</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>PA8</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>上拉输入</t>
+          <t>共地</t>
         </is>
       </c>
     </row>
     <row r="29" ht="8" customHeight="1">
-      <c r="A29" s="19" t="n"/>
+      <c r="A29" s="18" t="n"/>
       <c r="B29" s="11" t="n"/>
       <c r="C29" s="11" t="n"/>
       <c r="D29" s="11" t="n"/>
@@ -4460,50 +4202,266 @@
       <c r="G29" s="11" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>外接LED</t>
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>按键</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>状态LED</t>
+          <t>ID3(MSB)</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>PA15</t>
+          <t>PA0</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>PB5</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>门锁PA15/钥匙PB5</t>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="15" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>SW2</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>ID2</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>PC0</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="16" t="n"/>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>SW3</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>ID1</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>PC2</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="6" t="inlineStr"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>SW4</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ID0(LSB)</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>PC3</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="8" customHeight="1">
+      <c r="A34" s="17" t="n"/>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>按键</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>KEY-OK</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>确认</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>PA1</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="8" t="inlineStr"/>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>KEY-CANCEL</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>取消</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>PA8</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr"/>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>KEY-START</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>一键启动</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>PA0</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>上拉输入</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A4:A7"/>
-    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A30:A32"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:A12"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="A30"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A20:A23"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A14:A18"/>
     <mergeCell ref="A25:A28"/>
     <mergeCell ref="A19:G19"/>
   </mergeCells>
@@ -4517,315 +4475,267 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>引脚冲突解决对照表（屏幕不动方案）</t>
+          <t>LCD → OLED 方案变更说明</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>序号</t>
+          <t>变更项</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>冲突描述</t>
+          <t>LCD方案</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>涉及端</t>
+          <t>OLED方案</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>旧方案(有冲突)</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>新方案(已解决)</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
           <t>说明</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>PB0~PB15 = LCD数据总线 vs 板载LED</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>门锁端</t>
-        </is>
-      </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>LCD用PB0~PB15，LED也用PB0/PB1/PB5 → 冲突</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>放弃板载LED，外接LED到PA15</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>LCD必须用，LED改外接</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
+          <t>显示屏</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>ILI9341 LCD 16位8080并口</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>SSD1306/SH1106 OLED I2C</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>OLED只需2根线(SCL/SDA)，省14根数据线</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>PA9/PA10 = CH340(USART1) vs DL-20(USART1)</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>门锁端</t>
-        </is>
-      </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>DL-20和CH340都接USART1 → 冲突</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>DL-20改用软件串口(PA0/PA1)，CH340独占USART1</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>所有硬件USART已被占满，DL-20用软件串口9600</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
+          <t>占用引脚</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>PB0~PB15(数据)+PC4~PC7(控制)+PD2(背光)</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>PB6/PB7(I2C)+3.3V/GND</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>释放GPIOB全部16个引脚</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>PA0/PA1 = 拨码开关 vs 电容按键(TPAD)</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>门锁端</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>拨码开关用PA0/PA1，PA1有TPAD跳帽 → 冲突</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>拨码开关改到PC0/PC2/PC3/PA8，PA0/PA1给DL-20软件串口</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>PC0/PC2/PC3/PA8全部空闲</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
+          <t>触摸屏</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>XPT2046 模拟SPI(PC8~PC12)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>不需要</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>OLED通常不带触摸，改用按键交互</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>PC13 = 拨码开关 vs RTC晶振</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>门锁端</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>拨码开关用PC13，但PC13接RTC晶振</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>拨码开关不用PC13，改用PA8</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>PC13保留给RTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
+          <t>板载LED</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>PB0/PB1/PB5与LCD冲突不可用</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>PB0/PB1/PB5正常使用</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>GPIOB释放，LED无冲突</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>PC8~PC12 = 触摸屏 vs UART4/UART5</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>门锁端</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>触摸屏占PC8~PC12，UART4(PC10/11)/UART5(PC12)冲突</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>触摸屏不动，DL-20改软件串口不占UART</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>屏幕接线完全不动</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
+          <t>DL-20串口</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>软件串口PA0/PA1(9600)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>USART3 PB10/PB11(115200)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>GPIOB释放，可用硬件USART3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>PB0~PB15 = 钥匙端误标冲突</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>钥匙端</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>旧表标注"注意冲突"但钥匙端无LCD</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>标注"无冲突"，PB0/PB1/PB5正常用</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>钥匙端不接LCD</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+          <t>拨码开关</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>PC0/PC2/PC3/PA8</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>PA0/PC0/PC2/PC3</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>DL-20改USART3后PA0空闲，拨码开关用PA0更方便</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>PA9/PA10 = 钥匙端误标分时复用</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>钥匙端</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>旧表标注分时复用，但钥匙端无CH340</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>标注"无冲突"，DL-20独占USART1</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>钥匙端不需要CH340</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
+          <t>按键交互</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>无(用触摸屏)</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>PA1(确认)+PA8(取消)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>OLED无触摸，需外接按键</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>LQFP64封装PD口限制</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>两端</t>
-        </is>
-      </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>之前方案用PD3~PD15，但LQFP64只有PD0/PD1/PD2</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>全部改用PA/PC口，不依赖PD3~PD15</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>LQFP64仅51个GPIO</t>
+          <t>驱动代码</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>LCD驱动+触摸驱动复杂</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>OLED I2C驱动简单</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>SSD1306库广泛可用，代码量小</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>显示效果</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>320x240彩色</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>128x64单色/双色</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>OLED显示面积小，但对比度高、响应快</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>功耗</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>LCD+背光约150mA</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>OLED约20~30mA</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>OLED更省电</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4837,7 +4747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4872,12 +4782,12 @@
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>软件串口实现</t>
+          <t>OLED接线</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>门锁端DL-20用软件串口(PA0 TX / PA1 RX)，波特率9600。TX用Timer定时翻转GPIO，RX用外部中断下降沿触发+定时器采样。72MHz下9600波特率软件串口非常稳定。</t>
+          <t>SSD1306/SH1106 OLED使用I2C接口：PB6(SCL)、PB7(SDA)。I2C总线需要4.7k上拉电阻到3.3V。地址通常为0x78或0x7A。</t>
         </is>
       </c>
       <c r="C4" s="21" t="inlineStr">
@@ -4889,12 +4799,12 @@
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>屏幕接线不变</t>
+          <t>OLED库</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>LCD(ILI9341)和触摸屏(XPT2046)的接线完全保持原样，不需要修改任何现有驱动代码。PB0~PB15、PC4~PC7、PC8~PC12、PD2全部不动。</t>
+          <t>推荐使用开源SSD1306驱动库（如Adafruit_SSD1306或u8g2）。I2C配置：GPIO开漏输出+软件I2C或硬件I2C1。</t>
         </is>
       </c>
       <c r="C5" s="22" t="inlineStr">
@@ -4906,12 +4816,12 @@
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>USART资源分配</t>
+          <t>GPIOB释放</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>门锁端：USART1(CH340调试) + USART2(UWB基站) + 软件串口(DL-20)。钥匙端：USART1(DL-20) + USART2(UWB标签) + USART3(WiFi预留)。</t>
+          <t>放弃LCD后，GPIOB全部16个引脚(PB0~PB15)释放。板载LED(PB0绿/PB1蓝/PB5红)可正常使用。</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
@@ -4923,32 +4833,32 @@
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>拨码开关引脚</t>
+          <t>USART资源</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>门锁端4位拨码开关用PC0/PC2/PC3/PA8，全部是空闲引脚，无任何冲突。上拉输入，接GND=0，悬空=1。</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>门锁端：USART1(CH340调试) + USART2(UWB基站) + USART3(DL-20)。钥匙端：USART1(DL-20) + USART2(UWB标签) + USART3(WiFi预留)。全部硬件串口，无冲突。</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>LED方案</t>
+          <t>DL-20波特率</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>门锁端放弃板载LED(PB0/PB1/PB5与LCD冲突)，外接LED到PA15。需确保代码禁用JTAG(AFIO_Remap_SWJ_JTAGDisable)以释放PA15。钥匙端用PB5。</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
+          <t>门锁端DL-20改用USART3后可设115200（与UWB基站一致）。钥匙端USART1同样115200。</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -4957,32 +4867,32 @@
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>LQFP64封装限制</t>
+          <t>按键交互</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>STM32F103RCT6 LQFP64仅有PD0/PD1/PD2三个PD引脚，PD3~PD15不存在。所有外接功能必须用PA/PC口。</t>
-        </is>
-      </c>
-      <c r="C9" s="22" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>OLED不带触摸，门锁端需外接按键：PA1(确认/OK)、PA8(取消/CANCEL)。也可增加更多按键。</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>电源设计</t>
+          <t>拨码开关</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>门锁端USB 5V供电，板载AMS1117-3.3。钥匙端3.7V锂电池+AMS1117-3.3 LDO。</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
+          <t>门锁端4位拨码开关：PA0/PC0/PC2/PC3。PA0注意是一键启动按键的对端，不要混淆。</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -4991,29 +4901,29 @@
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>UWB基站配置</t>
+          <t>电源设计</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>GC-P2304-GS-2默认115200-8N1，数据格式：F0 06 ID_L ID_H DIST_L DIST_H ANGLE_L ANGLE_H RSSI AA。</t>
-        </is>
-      </c>
-      <c r="C11" s="22" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>门锁端USB 5V供电，板载AMS1117-3.3。钥匙端3.7V锂电池+AMS1117-3.3 LDO。OLED功耗约20~30mA。</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>UWB标签唤醒</t>
+          <t>UWB基站</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>GTM1000标签需要SOS脚(PB0)5ms高电平脉冲唤醒后才能UART透传，休眠电流&lt;40uA。</t>
+          <t>GC-P2304-GS-2默认115200-8N1，数据格式：F0 06 ID_L ID_H DIST_L DIST_H ANGLE_L ANGLE_H RSSI AA。</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
@@ -5025,12 +4935,12 @@
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>DL-20信道</t>
+          <t>UWB标签</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>门锁端和钥匙端DL-20需设置为相同信道(默认信道1)，建议点对点模式。门锁端波特率建议设9600(配合软件串口)。</t>
+          <t>GTM1000标签需要SOS脚(PB0)5ms高电平脉冲唤醒后才能UART透传，休眠电流&lt;40uA。</t>
         </is>
       </c>
       <c r="C13" s="22" t="inlineStr">
@@ -5042,12 +4952,12 @@
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>尺寸约束</t>
+          <t>DL-20信道</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>数字钥匙≤12×8×4cm，智能门锁≤直径60cm×高30cm圆柱体。</t>
+          <t>门锁端和钥匙端DL-20需设置为相同信道(默认信道1)，建议点对点模式。</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -5059,15 +4969,32 @@
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>尺寸约束</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>数字钥匙≤12×8×4cm，智能门锁≤直径60cm×高30cm圆柱体。</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
           <t>抗干扰</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>UWB天线附近不要铺地铜，远离电源和高频走线。DL-20天线尽量垂直放置。</t>
         </is>
       </c>
-      <c r="C15" s="22" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>高</t>
         </is>

</xml_diff>